<commit_message>
审计 Check list: 审计应对Checklist.xlsx
</commit_message>
<xml_diff>
--- a/审计应对Checklist.xlsx
+++ b/审计应对Checklist.xlsx
@@ -12,7 +12,7 @@
     <sheet name="③ 使用说明" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'① 逐项核对清单'!$A$1:$K$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'① 逐项核对清单'!$A$1:$M$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'② 按责任人派工'!$A$1:$I$168</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:M113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -550,7 +550,9 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -606,6 +608,16 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>更新人</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>更新时间</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>备注</t>
         </is>
       </c>
@@ -653,7 +665,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr"/>
+      <c r="K2" s="6" t="inlineStr"/>
+      <c r="L2" s="6" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -698,7 +712,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr"/>
+      <c r="L3" s="6" t="inlineStr"/>
+      <c r="M3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -743,7 +759,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr"/>
+      <c r="K4" s="6" t="inlineStr"/>
+      <c r="L4" s="6" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -788,7 +806,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -833,7 +853,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
+      <c r="L6" s="6" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -882,7 +904,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -931,7 +955,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr"/>
+      <c r="M8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -980,7 +1006,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1029,7 +1057,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
+      <c r="M10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1082,7 +1112,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
+      <c r="M11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1135,7 +1167,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
+      <c r="M12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1188,7 +1222,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr"/>
+      <c r="M13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1241,7 +1277,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr"/>
+      <c r="K14" s="6" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr"/>
+      <c r="M14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1294,7 +1332,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr"/>
+      <c r="M15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1347,7 +1387,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr"/>
+      <c r="K16" s="6" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr"/>
+      <c r="M16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1400,7 +1442,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr"/>
+      <c r="M17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1453,7 +1497,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr"/>
+      <c r="K18" s="6" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr"/>
+      <c r="M18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1506,7 +1552,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr"/>
+      <c r="K19" s="6" t="inlineStr"/>
+      <c r="L19" s="6" t="inlineStr"/>
+      <c r="M19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1559,7 +1607,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr"/>
+      <c r="K20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr"/>
+      <c r="M20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1612,7 +1662,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr"/>
+      <c r="K21" s="6" t="inlineStr"/>
+      <c r="L21" s="6" t="inlineStr"/>
+      <c r="M21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1665,7 +1717,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K22" s="5" t="inlineStr"/>
+      <c r="K22" s="6" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr"/>
+      <c r="M22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1714,7 +1768,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr"/>
+      <c r="K23" s="6" t="inlineStr"/>
+      <c r="L23" s="6" t="inlineStr"/>
+      <c r="M23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1763,7 +1819,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K24" s="5" t="inlineStr"/>
+      <c r="K24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr"/>
+      <c r="M24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1812,7 +1870,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K25" s="5" t="inlineStr"/>
+      <c r="K25" s="6" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr"/>
+      <c r="M25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1865,7 +1925,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K26" s="5" t="inlineStr"/>
+      <c r="K26" s="6" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr"/>
+      <c r="M26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1918,7 +1980,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K27" s="5" t="inlineStr"/>
+      <c r="K27" s="6" t="inlineStr"/>
+      <c r="L27" s="6" t="inlineStr"/>
+      <c r="M27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1971,7 +2035,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr"/>
+      <c r="K28" s="6" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr"/>
+      <c r="M28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2024,7 +2090,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K29" s="5" t="inlineStr"/>
+      <c r="K29" s="6" t="inlineStr"/>
+      <c r="L29" s="6" t="inlineStr"/>
+      <c r="M29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2077,7 +2145,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K30" s="5" t="inlineStr"/>
+      <c r="K30" s="6" t="inlineStr"/>
+      <c r="L30" s="6" t="inlineStr"/>
+      <c r="M30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -2130,7 +2200,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K31" s="5" t="inlineStr"/>
+      <c r="K31" s="6" t="inlineStr"/>
+      <c r="L31" s="6" t="inlineStr"/>
+      <c r="M31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -2183,7 +2255,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K32" s="5" t="inlineStr"/>
+      <c r="K32" s="6" t="inlineStr"/>
+      <c r="L32" s="6" t="inlineStr"/>
+      <c r="M32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -2228,7 +2302,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K33" s="5" t="inlineStr"/>
+      <c r="K33" s="6" t="inlineStr"/>
+      <c r="L33" s="6" t="inlineStr"/>
+      <c r="M33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -2273,7 +2349,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K34" s="5" t="inlineStr"/>
+      <c r="K34" s="6" t="inlineStr"/>
+      <c r="L34" s="6" t="inlineStr"/>
+      <c r="M34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2322,7 +2400,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K35" s="5" t="inlineStr"/>
+      <c r="K35" s="6" t="inlineStr"/>
+      <c r="L35" s="6" t="inlineStr"/>
+      <c r="M35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -2371,7 +2451,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K36" s="5" t="inlineStr"/>
+      <c r="K36" s="6" t="inlineStr"/>
+      <c r="L36" s="6" t="inlineStr"/>
+      <c r="M36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -2420,7 +2502,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K37" s="5" t="inlineStr"/>
+      <c r="K37" s="6" t="inlineStr"/>
+      <c r="L37" s="6" t="inlineStr"/>
+      <c r="M37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -2469,7 +2553,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K38" s="5" t="inlineStr"/>
+      <c r="K38" s="6" t="inlineStr"/>
+      <c r="L38" s="6" t="inlineStr"/>
+      <c r="M38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -2518,7 +2604,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K39" s="5" t="inlineStr"/>
+      <c r="K39" s="6" t="inlineStr"/>
+      <c r="L39" s="6" t="inlineStr"/>
+      <c r="M39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -2567,7 +2655,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K40" s="5" t="inlineStr"/>
+      <c r="K40" s="6" t="inlineStr"/>
+      <c r="L40" s="6" t="inlineStr"/>
+      <c r="M40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -2616,7 +2706,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K41" s="5" t="inlineStr"/>
+      <c r="K41" s="6" t="inlineStr"/>
+      <c r="L41" s="6" t="inlineStr"/>
+      <c r="M41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -2669,7 +2761,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K42" s="5" t="inlineStr"/>
+      <c r="K42" s="6" t="inlineStr"/>
+      <c r="L42" s="6" t="inlineStr"/>
+      <c r="M42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -2722,7 +2816,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K43" s="5" t="inlineStr"/>
+      <c r="K43" s="6" t="inlineStr"/>
+      <c r="L43" s="6" t="inlineStr"/>
+      <c r="M43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -2775,7 +2871,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K44" s="5" t="inlineStr"/>
+      <c r="K44" s="6" t="inlineStr"/>
+      <c r="L44" s="6" t="inlineStr"/>
+      <c r="M44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -2828,7 +2926,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K45" s="5" t="inlineStr"/>
+      <c r="K45" s="6" t="inlineStr"/>
+      <c r="L45" s="6" t="inlineStr"/>
+      <c r="M45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -2881,7 +2981,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K46" s="5" t="inlineStr"/>
+      <c r="K46" s="6" t="inlineStr"/>
+      <c r="L46" s="6" t="inlineStr"/>
+      <c r="M46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -2934,7 +3036,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K47" s="5" t="inlineStr"/>
+      <c r="K47" s="6" t="inlineStr"/>
+      <c r="L47" s="6" t="inlineStr"/>
+      <c r="M47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -2987,7 +3091,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K48" s="5" t="inlineStr"/>
+      <c r="K48" s="6" t="inlineStr"/>
+      <c r="L48" s="6" t="inlineStr"/>
+      <c r="M48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
@@ -3040,7 +3146,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K49" s="5" t="inlineStr"/>
+      <c r="K49" s="6" t="inlineStr"/>
+      <c r="L49" s="6" t="inlineStr"/>
+      <c r="M49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -3089,7 +3197,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K50" s="5" t="inlineStr"/>
+      <c r="K50" s="6" t="inlineStr"/>
+      <c r="L50" s="6" t="inlineStr"/>
+      <c r="M50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -3138,7 +3248,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K51" s="5" t="inlineStr"/>
+      <c r="K51" s="6" t="inlineStr"/>
+      <c r="L51" s="6" t="inlineStr"/>
+      <c r="M51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -3187,7 +3299,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K52" s="5" t="inlineStr"/>
+      <c r="K52" s="6" t="inlineStr"/>
+      <c r="L52" s="6" t="inlineStr"/>
+      <c r="M52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -3236,7 +3350,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K53" s="5" t="inlineStr"/>
+      <c r="K53" s="6" t="inlineStr"/>
+      <c r="L53" s="6" t="inlineStr"/>
+      <c r="M53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -3285,7 +3401,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K54" s="5" t="inlineStr"/>
+      <c r="K54" s="6" t="inlineStr"/>
+      <c r="L54" s="6" t="inlineStr"/>
+      <c r="M54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
@@ -3334,7 +3452,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K55" s="5" t="inlineStr"/>
+      <c r="K55" s="6" t="inlineStr"/>
+      <c r="L55" s="6" t="inlineStr"/>
+      <c r="M55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
@@ -3383,7 +3503,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K56" s="5" t="inlineStr"/>
+      <c r="K56" s="6" t="inlineStr"/>
+      <c r="L56" s="6" t="inlineStr"/>
+      <c r="M56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
@@ -3432,7 +3554,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K57" s="5" t="inlineStr"/>
+      <c r="K57" s="6" t="inlineStr"/>
+      <c r="L57" s="6" t="inlineStr"/>
+      <c r="M57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
@@ -3481,7 +3605,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K58" s="5" t="inlineStr"/>
+      <c r="K58" s="6" t="inlineStr"/>
+      <c r="L58" s="6" t="inlineStr"/>
+      <c r="M58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
@@ -3530,7 +3656,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K59" s="5" t="inlineStr"/>
+      <c r="K59" s="6" t="inlineStr"/>
+      <c r="L59" s="6" t="inlineStr"/>
+      <c r="M59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -3579,7 +3707,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K60" s="5" t="inlineStr"/>
+      <c r="K60" s="6" t="inlineStr"/>
+      <c r="L60" s="6" t="inlineStr"/>
+      <c r="M60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
@@ -3628,7 +3758,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K61" s="5" t="inlineStr"/>
+      <c r="K61" s="6" t="inlineStr"/>
+      <c r="L61" s="6" t="inlineStr"/>
+      <c r="M61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -3677,7 +3809,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K62" s="5" t="inlineStr"/>
+      <c r="K62" s="6" t="inlineStr"/>
+      <c r="L62" s="6" t="inlineStr"/>
+      <c r="M62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
@@ -3726,7 +3860,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K63" s="5" t="inlineStr"/>
+      <c r="K63" s="6" t="inlineStr"/>
+      <c r="L63" s="6" t="inlineStr"/>
+      <c r="M63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -3775,7 +3911,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K64" s="5" t="inlineStr"/>
+      <c r="K64" s="6" t="inlineStr"/>
+      <c r="L64" s="6" t="inlineStr"/>
+      <c r="M64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
@@ -3824,7 +3962,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K65" s="5" t="inlineStr"/>
+      <c r="K65" s="6" t="inlineStr"/>
+      <c r="L65" s="6" t="inlineStr"/>
+      <c r="M65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -3873,7 +4013,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K66" s="5" t="inlineStr"/>
+      <c r="K66" s="6" t="inlineStr"/>
+      <c r="L66" s="6" t="inlineStr"/>
+      <c r="M66" s="5" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
@@ -3922,7 +4064,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K67" s="5" t="inlineStr"/>
+      <c r="K67" s="6" t="inlineStr"/>
+      <c r="L67" s="6" t="inlineStr"/>
+      <c r="M67" s="5" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -3971,7 +4115,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K68" s="5" t="inlineStr"/>
+      <c r="K68" s="6" t="inlineStr"/>
+      <c r="L68" s="6" t="inlineStr"/>
+      <c r="M68" s="5" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
@@ -4020,7 +4166,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K69" s="5" t="inlineStr"/>
+      <c r="K69" s="6" t="inlineStr"/>
+      <c r="L69" s="6" t="inlineStr"/>
+      <c r="M69" s="5" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -4069,7 +4217,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K70" s="5" t="inlineStr"/>
+      <c r="K70" s="6" t="inlineStr"/>
+      <c r="L70" s="6" t="inlineStr"/>
+      <c r="M70" s="5" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
@@ -4118,7 +4268,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K71" s="5" t="inlineStr"/>
+      <c r="K71" s="6" t="inlineStr"/>
+      <c r="L71" s="6" t="inlineStr"/>
+      <c r="M71" s="5" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -4167,7 +4319,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K72" s="5" t="inlineStr"/>
+      <c r="K72" s="6" t="inlineStr"/>
+      <c r="L72" s="6" t="inlineStr"/>
+      <c r="M72" s="5" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
@@ -4216,7 +4370,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K73" s="5" t="inlineStr"/>
+      <c r="K73" s="6" t="inlineStr"/>
+      <c r="L73" s="6" t="inlineStr"/>
+      <c r="M73" s="5" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
@@ -4261,7 +4417,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K74" s="5" t="inlineStr"/>
+      <c r="K74" s="6" t="inlineStr"/>
+      <c r="L74" s="6" t="inlineStr"/>
+      <c r="M74" s="5" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
@@ -4306,7 +4464,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K75" s="5" t="inlineStr"/>
+      <c r="K75" s="6" t="inlineStr"/>
+      <c r="L75" s="6" t="inlineStr"/>
+      <c r="M75" s="5" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4351,7 +4511,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K76" s="5" t="inlineStr"/>
+      <c r="K76" s="6" t="inlineStr"/>
+      <c r="L76" s="6" t="inlineStr"/>
+      <c r="M76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
@@ -4396,7 +4558,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K77" s="5" t="inlineStr"/>
+      <c r="K77" s="6" t="inlineStr"/>
+      <c r="L77" s="6" t="inlineStr"/>
+      <c r="M77" s="5" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -4445,7 +4609,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K78" s="5" t="inlineStr"/>
+      <c r="K78" s="6" t="inlineStr"/>
+      <c r="L78" s="6" t="inlineStr"/>
+      <c r="M78" s="5" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
@@ -4494,7 +4660,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K79" s="5" t="inlineStr"/>
+      <c r="K79" s="6" t="inlineStr"/>
+      <c r="L79" s="6" t="inlineStr"/>
+      <c r="M79" s="5" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
@@ -4543,7 +4711,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K80" s="5" t="inlineStr"/>
+      <c r="K80" s="6" t="inlineStr"/>
+      <c r="L80" s="6" t="inlineStr"/>
+      <c r="M80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4596,7 +4766,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K81" s="5" t="inlineStr"/>
+      <c r="K81" s="6" t="inlineStr"/>
+      <c r="L81" s="6" t="inlineStr"/>
+      <c r="M81" s="5" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
@@ -4649,7 +4821,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K82" s="5" t="inlineStr"/>
+      <c r="K82" s="6" t="inlineStr"/>
+      <c r="L82" s="6" t="inlineStr"/>
+      <c r="M82" s="5" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
@@ -4702,7 +4876,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K83" s="5" t="inlineStr"/>
+      <c r="K83" s="6" t="inlineStr"/>
+      <c r="L83" s="6" t="inlineStr"/>
+      <c r="M83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -4747,7 +4923,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K84" s="5" t="inlineStr"/>
+      <c r="K84" s="6" t="inlineStr"/>
+      <c r="L84" s="6" t="inlineStr"/>
+      <c r="M84" s="5" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
@@ -4796,7 +4974,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K85" s="5" t="inlineStr"/>
+      <c r="K85" s="6" t="inlineStr"/>
+      <c r="L85" s="6" t="inlineStr"/>
+      <c r="M85" s="5" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
@@ -4841,7 +5021,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K86" s="5" t="inlineStr"/>
+      <c r="K86" s="6" t="inlineStr"/>
+      <c r="L86" s="6" t="inlineStr"/>
+      <c r="M86" s="5" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
@@ -4890,7 +5072,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K87" s="5" t="inlineStr"/>
+      <c r="K87" s="6" t="inlineStr"/>
+      <c r="L87" s="6" t="inlineStr"/>
+      <c r="M87" s="5" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
@@ -4935,7 +5119,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K88" s="5" t="inlineStr"/>
+      <c r="K88" s="6" t="inlineStr"/>
+      <c r="L88" s="6" t="inlineStr"/>
+      <c r="M88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
@@ -4980,7 +5166,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K89" s="5" t="inlineStr"/>
+      <c r="K89" s="6" t="inlineStr"/>
+      <c r="L89" s="6" t="inlineStr"/>
+      <c r="M89" s="5" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5033,7 +5221,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K90" s="5" t="inlineStr"/>
+      <c r="K90" s="6" t="inlineStr"/>
+      <c r="L90" s="6" t="inlineStr"/>
+      <c r="M90" s="5" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
@@ -5086,7 +5276,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K91" s="5" t="inlineStr"/>
+      <c r="K91" s="6" t="inlineStr"/>
+      <c r="L91" s="6" t="inlineStr"/>
+      <c r="M91" s="5" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
@@ -5139,7 +5331,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K92" s="5" t="inlineStr"/>
+      <c r="K92" s="6" t="inlineStr"/>
+      <c r="L92" s="6" t="inlineStr"/>
+      <c r="M92" s="5" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
@@ -5192,7 +5386,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K93" s="5" t="inlineStr"/>
+      <c r="K93" s="6" t="inlineStr"/>
+      <c r="L93" s="6" t="inlineStr"/>
+      <c r="M93" s="5" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
@@ -5245,7 +5441,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K94" s="5" t="inlineStr"/>
+      <c r="K94" s="6" t="inlineStr"/>
+      <c r="L94" s="6" t="inlineStr"/>
+      <c r="M94" s="5" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
@@ -5298,7 +5496,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K95" s="5" t="inlineStr"/>
+      <c r="K95" s="6" t="inlineStr"/>
+      <c r="L95" s="6" t="inlineStr"/>
+      <c r="M95" s="5" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
@@ -5351,7 +5551,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K96" s="5" t="inlineStr"/>
+      <c r="K96" s="6" t="inlineStr"/>
+      <c r="L96" s="6" t="inlineStr"/>
+      <c r="M96" s="5" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
@@ -5404,7 +5606,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K97" s="5" t="inlineStr"/>
+      <c r="K97" s="6" t="inlineStr"/>
+      <c r="L97" s="6" t="inlineStr"/>
+      <c r="M97" s="5" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
@@ -5457,7 +5661,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K98" s="5" t="inlineStr"/>
+      <c r="K98" s="6" t="inlineStr"/>
+      <c r="L98" s="6" t="inlineStr"/>
+      <c r="M98" s="5" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
@@ -5506,7 +5712,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K99" s="5" t="inlineStr"/>
+      <c r="K99" s="6" t="inlineStr"/>
+      <c r="L99" s="6" t="inlineStr"/>
+      <c r="M99" s="5" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5551,7 +5759,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K100" s="5" t="inlineStr"/>
+      <c r="K100" s="6" t="inlineStr"/>
+      <c r="L100" s="6" t="inlineStr"/>
+      <c r="M100" s="5" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
@@ -5596,7 +5806,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K101" s="5" t="inlineStr"/>
+      <c r="K101" s="6" t="inlineStr"/>
+      <c r="L101" s="6" t="inlineStr"/>
+      <c r="M101" s="5" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
@@ -5641,7 +5853,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K102" s="5" t="inlineStr"/>
+      <c r="K102" s="6" t="inlineStr"/>
+      <c r="L102" s="6" t="inlineStr"/>
+      <c r="M102" s="5" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -5690,7 +5904,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K103" s="5" t="inlineStr"/>
+      <c r="K103" s="6" t="inlineStr"/>
+      <c r="L103" s="6" t="inlineStr"/>
+      <c r="M103" s="5" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
@@ -5735,7 +5951,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K104" s="5" t="inlineStr"/>
+      <c r="K104" s="6" t="inlineStr"/>
+      <c r="L104" s="6" t="inlineStr"/>
+      <c r="M104" s="5" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
@@ -5780,7 +5998,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K105" s="5" t="inlineStr"/>
+      <c r="K105" s="6" t="inlineStr"/>
+      <c r="L105" s="6" t="inlineStr"/>
+      <c r="M105" s="5" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
@@ -5825,7 +6045,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K106" s="5" t="inlineStr"/>
+      <c r="K106" s="6" t="inlineStr"/>
+      <c r="L106" s="6" t="inlineStr"/>
+      <c r="M106" s="5" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
@@ -5874,7 +6096,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K107" s="5" t="inlineStr"/>
+      <c r="K107" s="6" t="inlineStr"/>
+      <c r="L107" s="6" t="inlineStr"/>
+      <c r="M107" s="5" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
@@ -5919,7 +6143,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K108" s="5" t="inlineStr"/>
+      <c r="K108" s="6" t="inlineStr"/>
+      <c r="L108" s="6" t="inlineStr"/>
+      <c r="M108" s="5" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
@@ -5964,7 +6190,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K109" s="5" t="inlineStr"/>
+      <c r="K109" s="6" t="inlineStr"/>
+      <c r="L109" s="6" t="inlineStr"/>
+      <c r="M109" s="5" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
@@ -6009,7 +6237,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K110" s="5" t="inlineStr"/>
+      <c r="K110" s="6" t="inlineStr"/>
+      <c r="L110" s="6" t="inlineStr"/>
+      <c r="M110" s="5" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
@@ -6054,7 +6284,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K111" s="5" t="inlineStr"/>
+      <c r="K111" s="6" t="inlineStr"/>
+      <c r="L111" s="6" t="inlineStr"/>
+      <c r="M111" s="5" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
@@ -6099,7 +6331,9 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K112" s="5" t="inlineStr"/>
+      <c r="K112" s="6" t="inlineStr"/>
+      <c r="L112" s="6" t="inlineStr"/>
+      <c r="M112" s="5" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
@@ -6144,10 +6378,12 @@
           <t>未开始</t>
         </is>
       </c>
-      <c r="K113" s="5" t="inlineStr"/>
+      <c r="K113" s="6" t="inlineStr"/>
+      <c r="L113" s="6" t="inlineStr"/>
+      <c r="M113" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K113"/>
+  <autoFilter ref="A1:M113"/>
   <dataValidations count="2">
     <dataValidation sqref="J2:J113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="请从下拉列表选择" prompt="未开始 / 准备中 / 已就绪 / 不适用" type="list">
       <formula1>"未开始,准备中,已就绪,不适用"</formula1>

</xml_diff>